<commit_message>
fix(excel): _find_table_bounds fix for #2626
</commit_message>
<xml_diff>
--- a/tests/data/xlsx/xlsx_06_table_with_missing_headers_tail.xlsx
+++ b/tests/data/xlsx/xlsx_06_table_with_missing_headers_tail.xlsx
@@ -470,7 +470,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K16"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16.5"/>
@@ -482,112 +482,92 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0"/>
-      <c r="B1" s="0"/>
-      <c r="C1" s="0"/>
-      <c r="D1" s="0"/>
-      <c r="E1" s="0"/>
-      <c r="F1" s="0"/>
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0"/>
-      <c r="B2" s="0"/>
-      <c r="C2" s="0"/>
-      <c r="D2" s="0"/>
-      <c r="E2" s="0"/>
-      <c r="F2" s="0"/>
+      <c r="A2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0"/>
-      <c r="B3" s="0"/>
-      <c r="C3" s="0"/>
-      <c r="D3" s="0"/>
-      <c r="E3" s="0"/>
-      <c r="F3" s="0"/>
+      <c r="A3" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0"/>
-      <c r="B4" s="0"/>
-      <c r="C4" s="0"/>
-      <c r="D4" s="0"/>
-      <c r="E4" s="0"/>
-      <c r="F4" s="0"/>
+      <c r="A4" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="F13" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="I13" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="J13" s="2"/>
-      <c r="K13" s="2"/>
+      <c r="F13" s="0"/>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="F14" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="I14" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="J14" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="K14" s="4" t="s">
-        <v>9</v>
-      </c>
+      <c r="F14" s="0"/>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="F15" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="G15" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="H15" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="I15" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="J15" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="K15" s="5" t="s">
-        <v>13</v>
-      </c>
+      <c r="F15" s="0"/>
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="F16" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="H16" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="I16" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="J16" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="K16" s="3" t="s">
-        <v>17</v>
-      </c>
+      <c r="F16" s="0"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>